<commit_message>
new run results ;)
</commit_message>
<xml_diff>
--- a/ttp_literature_catABC_results_updated.xlsx
+++ b/ttp_literature_catABC_results_updated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maohammed/Documents/Applied AI Master/Level 4/Graudition research/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maohammed/Desktop/ttp-dashboard-repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04924FAE-4AAD-5A41-A9D5-AD03BEDA08D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7958396B-C328-E545-867E-BAF4A45692F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="-6100" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="-5500" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instances CatA,B,C" sheetId="4" r:id="rId1"/>
@@ -492,7 +492,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -512,12 +512,6 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -982,7 +976,7 @@
     <col min="19" max="19" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="64" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>134</v>
       </c>
@@ -1041,7 +1035,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1138,7 +1132,7 @@
         <v>3717</v>
       </c>
       <c r="S3" s="8">
-        <v>3869.46</v>
+        <v>3776.88</v>
       </c>
       <c r="T3" s="16"/>
     </row>
@@ -1198,7 +1192,7 @@
         <v>4703</v>
       </c>
       <c r="S4" s="8">
-        <v>4510.99</v>
+        <v>4610.6400000000003</v>
       </c>
       <c r="T4" s="16"/>
     </row>
@@ -1258,7 +1252,7 @@
         <v>8868</v>
       </c>
       <c r="S5" s="8">
-        <v>8430.1</v>
+        <v>9291.42</v>
       </c>
     </row>
     <row r="6" spans="1:24" ht="16" x14ac:dyDescent="0.2">
@@ -1317,7 +1311,7 @@
         <v>8314</v>
       </c>
       <c r="S6" s="8">
-        <v>8643.33</v>
+        <v>8678.73</v>
       </c>
       <c r="T6" s="17"/>
     </row>
@@ -1377,7 +1371,7 @@
         <v>17639</v>
       </c>
       <c r="S7" s="8">
-        <v>16666.150000000001</v>
+        <v>18572.2</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="16" x14ac:dyDescent="0.2">
@@ -1436,7 +1430,7 @@
         <v>25881</v>
       </c>
       <c r="S8" s="8">
-        <v>26933.64</v>
+        <v>27014.82</v>
       </c>
       <c r="T8" s="17"/>
     </row>
@@ -1496,7 +1490,7 @@
         <v>48865</v>
       </c>
       <c r="S9" s="8">
-        <v>49152.97</v>
+        <v>49852.63</v>
       </c>
     </row>
     <row r="10" spans="1:24" ht="16" x14ac:dyDescent="0.2">
@@ -1619,7 +1613,7 @@
         <v>75804</v>
       </c>
       <c r="S11" s="8">
-        <v>77508.149999999994</v>
+        <v>79782.44</v>
       </c>
       <c r="T11" s="17"/>
       <c r="W11" s="19" t="s">
@@ -1683,7 +1677,7 @@
         <v>88330</v>
       </c>
       <c r="S12" s="8">
-        <v>76897.64</v>
+        <v>90840.44</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="16" x14ac:dyDescent="0.2">
@@ -1742,7 +1736,7 @@
         <v>112686</v>
       </c>
       <c r="S13" s="8">
-        <v>117720.46</v>
+        <v>120280.22</v>
       </c>
       <c r="T13" s="16"/>
     </row>
@@ -1802,7 +1796,7 @@
         <v>148988</v>
       </c>
       <c r="S14" s="8">
-        <v>156834.21</v>
+        <v>158354.07999999999</v>
       </c>
       <c r="T14" s="17"/>
     </row>
@@ -1862,7 +1856,7 @@
         <v>248482</v>
       </c>
       <c r="S15" s="8">
-        <v>257267.54</v>
+        <v>259229.62</v>
       </c>
       <c r="T15" s="17"/>
     </row>
@@ -1922,7 +1916,7 @@
         <v>367247</v>
       </c>
       <c r="S16" s="8">
-        <v>290589.18</v>
+        <v>357038.4</v>
       </c>
     </row>
     <row r="17" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -1981,7 +1975,7 @@
         <v>662940</v>
       </c>
       <c r="S17" s="8">
-        <v>695074.34</v>
+        <v>702907.69</v>
       </c>
       <c r="T17" s="17"/>
     </row>
@@ -2041,7 +2035,7 @@
         <v>743146</v>
       </c>
       <c r="S18" s="8">
-        <v>647297.6</v>
+        <v>796257.45</v>
       </c>
     </row>
     <row r="19" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2100,7 +2094,7 @@
         <v>813977</v>
       </c>
       <c r="S19" s="8">
-        <v>856742.35</v>
+        <v>862903.49</v>
       </c>
       <c r="T19" s="17"/>
     </row>
@@ -2160,7 +2154,7 @@
         <v>871348</v>
       </c>
       <c r="S20" s="8">
-        <v>924699.62</v>
+        <v>926449.25</v>
       </c>
       <c r="T20" s="17"/>
     </row>
@@ -2220,7 +2214,7 @@
         <v>996820</v>
       </c>
       <c r="S21" s="8">
-        <v>1051087.8</v>
+        <v>1062026.5</v>
       </c>
       <c r="T21" s="17"/>
     </row>
@@ -2280,7 +2274,7 @@
         <v>1730997</v>
       </c>
       <c r="S22" s="8">
-        <v>1748837.31</v>
+        <v>1864553.19</v>
       </c>
       <c r="T22" s="16"/>
     </row>
@@ -2340,7 +2334,7 @@
         <v>22286</v>
       </c>
       <c r="S23" s="12">
-        <v>21061.07</v>
+        <v>21149.54</v>
       </c>
       <c r="T23" s="16"/>
     </row>
@@ -2400,7 +2394,7 @@
         <v>43310</v>
       </c>
       <c r="S24" s="12">
-        <v>45436.71</v>
+        <v>44029.34</v>
       </c>
       <c r="T24" s="17"/>
     </row>
@@ -2460,7 +2454,7 @@
         <v>60705</v>
       </c>
       <c r="S25" s="12">
-        <v>51581.31</v>
+        <v>57419.77</v>
       </c>
       <c r="T25" s="16"/>
     </row>
@@ -2520,7 +2514,7 @@
         <v>58778</v>
       </c>
       <c r="S26" s="12">
-        <v>56629.03</v>
+        <v>57752.5</v>
       </c>
     </row>
     <row r="27" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2579,7 +2573,7 @@
         <v>111728</v>
       </c>
       <c r="S27" s="12">
-        <v>108522.03</v>
+        <v>111223.67</v>
       </c>
       <c r="T27" s="16"/>
     </row>
@@ -2639,7 +2633,7 @@
         <v>252294</v>
       </c>
       <c r="S28" s="12">
-        <v>230979.21</v>
+        <v>247464.62</v>
       </c>
     </row>
     <row r="29" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2698,7 +2692,7 @@
         <v>303046</v>
       </c>
       <c r="S29" s="12">
-        <v>286291.25</v>
+        <v>304004.06</v>
       </c>
     </row>
     <row r="30" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2757,7 +2751,7 @@
         <v>339630</v>
       </c>
       <c r="S30" s="12">
-        <v>324979.71999999997</v>
+        <v>298413.65000000002</v>
       </c>
     </row>
     <row r="31" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2816,7 +2810,7 @@
         <v>573980</v>
       </c>
       <c r="S31" s="12">
-        <v>558243.62</v>
+        <v>565861.19999999995</v>
       </c>
     </row>
     <row r="32" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2875,7 +2869,7 @@
         <v>603443</v>
       </c>
       <c r="S32" s="12">
-        <v>385244.12</v>
+        <v>597593.44999999995</v>
       </c>
     </row>
     <row r="33" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2934,7 +2928,7 @@
         <v>842566</v>
       </c>
       <c r="S33" s="12">
-        <v>797985.94</v>
+        <v>823863.77</v>
       </c>
     </row>
     <row r="34" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2993,7 +2987,7 @@
         <v>1164547</v>
       </c>
       <c r="S34" s="12">
-        <v>1077239.43</v>
+        <v>1095981.6499999999</v>
       </c>
     </row>
     <row r="35" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3052,7 +3046,7 @@
         <v>1616072</v>
       </c>
       <c r="S35" s="12">
-        <v>1485261.81</v>
+        <v>1489376.46</v>
       </c>
     </row>
     <row r="36" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3111,7 +3105,7 @@
         <v>4248266</v>
       </c>
       <c r="S36" s="12">
-        <v>2941686.19</v>
+        <v>4130947.76</v>
       </c>
     </row>
     <row r="37" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3170,7 +3164,7 @@
         <v>4583308</v>
       </c>
       <c r="S37" s="12">
-        <v>4282123.22</v>
+        <v>4248811.8099999996</v>
       </c>
     </row>
     <row r="38" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3229,7 +3223,7 @@
         <v>7770907</v>
       </c>
       <c r="S38" s="12">
-        <v>5239874.4800000004</v>
+        <v>7916822.1100000003</v>
       </c>
     </row>
     <row r="39" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3288,7 +3282,7 @@
         <v>6467038</v>
       </c>
       <c r="S39" s="12">
-        <v>6244168.29</v>
+        <v>6249284.3799999999</v>
       </c>
     </row>
     <row r="40" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3347,7 +3341,7 @@
         <v>6797757</v>
       </c>
       <c r="S40" s="12">
-        <v>6377272.4699999997</v>
+        <v>7123429.2599999998</v>
       </c>
     </row>
     <row r="41" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3406,7 +3400,7 @@
         <v>7102985</v>
       </c>
       <c r="S41" s="12">
-        <v>6638110.8700000001</v>
+        <v>7020979.2699999996</v>
       </c>
     </row>
     <row r="42" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3465,7 +3459,7 @@
         <v>15605360</v>
       </c>
       <c r="S42" s="12">
-        <v>14098365.16</v>
+        <v>14724194.82</v>
       </c>
     </row>
     <row r="43" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3524,7 +3518,7 @@
         <v>88131</v>
       </c>
       <c r="S43" s="10">
-        <v>86398.9</v>
+        <v>86365.67</v>
       </c>
     </row>
     <row r="44" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3583,7 +3577,7 @@
         <v>155500</v>
       </c>
       <c r="S44" s="10">
-        <v>155630.14000000001</v>
+        <v>155630.15</v>
       </c>
       <c r="T44" s="16"/>
     </row>
@@ -3643,7 +3637,7 @@
         <v>205552</v>
       </c>
       <c r="S45" s="10">
-        <v>193429.5</v>
+        <v>206388.68</v>
       </c>
     </row>
     <row r="46" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3702,7 +3696,7 @@
         <v>242452</v>
       </c>
       <c r="S46" s="10">
-        <v>242278.37</v>
+        <v>243568.75</v>
       </c>
       <c r="T46" s="16"/>
     </row>
@@ -3762,7 +3756,7 @@
         <v>426951</v>
       </c>
       <c r="S47" s="10">
-        <v>410325.89</v>
+        <v>425482.95</v>
       </c>
     </row>
     <row r="48" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3821,7 +3815,7 @@
         <v>969064</v>
       </c>
       <c r="S48" s="10">
-        <v>929720.5</v>
+        <v>961153.43</v>
       </c>
     </row>
     <row r="49" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3880,7 +3874,7 @@
         <v>1187092</v>
       </c>
       <c r="S49" s="10">
-        <v>1155115.81</v>
+        <v>1187092.5900000001</v>
       </c>
     </row>
     <row r="50" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3939,7 +3933,7 @@
         <v>1442153</v>
       </c>
       <c r="S50" s="10">
-        <v>1419472.61</v>
+        <v>1466642.54</v>
       </c>
     </row>
     <row r="51" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3998,7 +3992,7 @@
         <v>2183137</v>
       </c>
       <c r="S51" s="10">
-        <v>2153426.0099999998</v>
+        <v>2173578.39</v>
       </c>
     </row>
     <row r="52" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4057,7 +4051,7 @@
         <v>2470833</v>
       </c>
       <c r="S52" s="10">
-        <v>1848666.67</v>
+        <v>2398853.48</v>
       </c>
     </row>
     <row r="53" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4116,7 +4110,7 @@
         <v>3399342</v>
       </c>
       <c r="S53" s="10">
-        <v>3203138.48</v>
+        <v>3336058.43</v>
       </c>
     </row>
     <row r="54" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4175,7 +4169,7 @@
         <v>4553407</v>
       </c>
       <c r="S54" s="10">
-        <v>4559461.8</v>
+        <v>4570523.9800000004</v>
       </c>
       <c r="T54" s="16"/>
     </row>
@@ -4235,7 +4229,7 @@
         <v>6552392</v>
       </c>
       <c r="S55" s="10">
-        <v>6458049.9100000001</v>
+        <v>6520606.3700000001</v>
       </c>
     </row>
     <row r="56" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4294,7 +4288,7 @@
         <v>13891830</v>
       </c>
       <c r="S56" s="10">
-        <v>10943665.23</v>
+        <v>13816880.529999999</v>
       </c>
     </row>
     <row r="57" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4353,7 +4347,7 @@
         <v>18273340</v>
       </c>
       <c r="S57" s="10">
-        <v>17255072.239999998</v>
+        <v>18026388.100000001</v>
       </c>
     </row>
     <row r="58" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4412,7 +4406,7 @@
         <v>26010780</v>
       </c>
       <c r="S58" s="10">
-        <v>22153339.030000001</v>
+        <v>26029479.48</v>
       </c>
     </row>
     <row r="59" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4471,7 +4465,7 @@
         <v>23687540</v>
       </c>
       <c r="S59" s="10">
-        <v>22998344.649999999</v>
+        <v>23583861.52</v>
       </c>
     </row>
     <row r="60" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4530,7 +4524,7 @@
         <v>26032000</v>
       </c>
       <c r="S60" s="10">
-        <v>23337446.949999999</v>
+        <v>26807644.57</v>
       </c>
     </row>
     <row r="61" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4589,7 +4583,7 @@
         <v>27282770</v>
       </c>
       <c r="S61" s="10">
-        <v>25958966.460000001</v>
+        <v>27334035.09</v>
       </c>
     </row>
     <row r="62" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4648,7 +4642,7 @@
         <v>57896250</v>
       </c>
       <c r="S62" s="10">
-        <v>51058556.299999997</v>
+        <v>56748874.119999997</v>
       </c>
     </row>
     <row r="63" spans="1:20" ht="16" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
New results for my MMAILS ;)
</commit_message>
<xml_diff>
--- a/ttp_literature_catABC_results_updated.xlsx
+++ b/ttp_literature_catABC_results_updated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maohammed/Desktop/ttp-dashboard-repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7958396B-C328-E545-867E-BAF4A45692F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F0C1D8-BB4D-BC4A-AFFC-C83C71754838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38400" yWindow="-5500" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1132,7 +1132,7 @@
         <v>3717</v>
       </c>
       <c r="S3" s="8">
-        <v>3776.88</v>
+        <v>4100.8</v>
       </c>
       <c r="T3" s="16"/>
     </row>
@@ -1192,7 +1192,7 @@
         <v>4703</v>
       </c>
       <c r="S4" s="8">
-        <v>4610.6400000000003</v>
+        <v>4911.16</v>
       </c>
       <c r="T4" s="16"/>
     </row>
@@ -1252,7 +1252,7 @@
         <v>8868</v>
       </c>
       <c r="S5" s="8">
-        <v>9291.42</v>
+        <v>9680.64</v>
       </c>
     </row>
     <row r="6" spans="1:24" ht="16" x14ac:dyDescent="0.2">
@@ -1311,7 +1311,7 @@
         <v>8314</v>
       </c>
       <c r="S6" s="8">
-        <v>8678.73</v>
+        <v>9063.68</v>
       </c>
       <c r="T6" s="17"/>
     </row>
@@ -1371,7 +1371,7 @@
         <v>17639</v>
       </c>
       <c r="S7" s="8">
-        <v>18572.2</v>
+        <v>19164.439999999999</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="16" x14ac:dyDescent="0.2">
@@ -1430,7 +1430,7 @@
         <v>25881</v>
       </c>
       <c r="S8" s="8">
-        <v>27014.82</v>
+        <v>28195.53</v>
       </c>
       <c r="T8" s="17"/>
     </row>
@@ -1490,7 +1490,7 @@
         <v>48865</v>
       </c>
       <c r="S9" s="8">
-        <v>49852.63</v>
+        <v>50872.11</v>
       </c>
     </row>
     <row r="10" spans="1:24" ht="16" x14ac:dyDescent="0.2">
@@ -1549,7 +1549,7 @@
         <v>143699</v>
       </c>
       <c r="S10" s="8">
-        <v>144219</v>
+        <v>144426</v>
       </c>
       <c r="T10" s="17"/>
       <c r="W10" s="18" t="s">
@@ -1613,7 +1613,7 @@
         <v>75804</v>
       </c>
       <c r="S11" s="8">
-        <v>79782.44</v>
+        <v>81660.87</v>
       </c>
       <c r="T11" s="17"/>
       <c r="W11" s="19" t="s">
@@ -1677,7 +1677,7 @@
         <v>88330</v>
       </c>
       <c r="S12" s="8">
-        <v>90840.44</v>
+        <v>92517.04</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="16" x14ac:dyDescent="0.2">
@@ -1736,7 +1736,7 @@
         <v>112686</v>
       </c>
       <c r="S13" s="8">
-        <v>120280.22</v>
+        <v>120744.83</v>
       </c>
       <c r="T13" s="16"/>
     </row>
@@ -1796,7 +1796,7 @@
         <v>148988</v>
       </c>
       <c r="S14" s="8">
-        <v>158354.07999999999</v>
+        <v>161191.96</v>
       </c>
       <c r="T14" s="17"/>
     </row>
@@ -1856,7 +1856,7 @@
         <v>248482</v>
       </c>
       <c r="S15" s="8">
-        <v>259229.62</v>
+        <v>263543.98</v>
       </c>
       <c r="T15" s="17"/>
     </row>
@@ -1916,7 +1916,7 @@
         <v>367247</v>
       </c>
       <c r="S16" s="8">
-        <v>357038.4</v>
+        <v>403684.62</v>
       </c>
     </row>
     <row r="17" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -1975,7 +1975,7 @@
         <v>662940</v>
       </c>
       <c r="S17" s="8">
-        <v>702907.69</v>
+        <v>710997.64</v>
       </c>
       <c r="T17" s="17"/>
     </row>
@@ -2035,7 +2035,7 @@
         <v>743146</v>
       </c>
       <c r="S18" s="8">
-        <v>796257.45</v>
+        <v>810879.96</v>
       </c>
     </row>
     <row r="19" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2094,7 +2094,7 @@
         <v>813977</v>
       </c>
       <c r="S19" s="8">
-        <v>862903.49</v>
+        <v>873102.07</v>
       </c>
       <c r="T19" s="17"/>
     </row>
@@ -2154,7 +2154,7 @@
         <v>871348</v>
       </c>
       <c r="S20" s="8">
-        <v>926449.25</v>
+        <v>952282.51</v>
       </c>
       <c r="T20" s="17"/>
     </row>
@@ -2214,7 +2214,7 @@
         <v>996820</v>
       </c>
       <c r="S21" s="8">
-        <v>1062026.5</v>
+        <v>1078267.3799999999</v>
       </c>
       <c r="T21" s="17"/>
     </row>
@@ -2274,7 +2274,7 @@
         <v>1730997</v>
       </c>
       <c r="S22" s="8">
-        <v>1864553.19</v>
+        <v>1917935.56</v>
       </c>
       <c r="T22" s="16"/>
     </row>
@@ -2334,7 +2334,7 @@
         <v>22286</v>
       </c>
       <c r="S23" s="12">
-        <v>21149.54</v>
+        <v>22776.92</v>
       </c>
       <c r="T23" s="16"/>
     </row>
@@ -2394,7 +2394,7 @@
         <v>43310</v>
       </c>
       <c r="S24" s="12">
-        <v>44029.34</v>
+        <v>46633.18</v>
       </c>
       <c r="T24" s="17"/>
     </row>
@@ -2454,7 +2454,7 @@
         <v>60705</v>
       </c>
       <c r="S25" s="12">
-        <v>57419.77</v>
+        <v>61718.36</v>
       </c>
       <c r="T25" s="16"/>
     </row>
@@ -2514,7 +2514,7 @@
         <v>58778</v>
       </c>
       <c r="S26" s="12">
-        <v>57752.5</v>
+        <v>61563.32</v>
       </c>
     </row>
     <row r="27" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2573,7 +2573,7 @@
         <v>111728</v>
       </c>
       <c r="S27" s="12">
-        <v>111223.67</v>
+        <v>111443.25</v>
       </c>
       <c r="T27" s="16"/>
     </row>
@@ -2633,7 +2633,7 @@
         <v>252294</v>
       </c>
       <c r="S28" s="12">
-        <v>247464.62</v>
+        <v>254878.9</v>
       </c>
     </row>
     <row r="29" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2692,7 +2692,7 @@
         <v>303046</v>
       </c>
       <c r="S29" s="12">
-        <v>304004.06</v>
+        <v>317580.79999999999</v>
       </c>
     </row>
     <row r="30" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2751,7 +2751,7 @@
         <v>339630</v>
       </c>
       <c r="S30" s="12">
-        <v>298413.65000000002</v>
+        <v>350166.13</v>
       </c>
     </row>
     <row r="31" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2810,7 +2810,7 @@
         <v>573980</v>
       </c>
       <c r="S31" s="12">
-        <v>565861.19999999995</v>
+        <v>594322.31999999995</v>
       </c>
     </row>
     <row r="32" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2869,7 +2869,7 @@
         <v>603443</v>
       </c>
       <c r="S32" s="12">
-        <v>597593.44999999995</v>
+        <v>613270.18000000005</v>
       </c>
     </row>
     <row r="33" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2928,7 +2928,7 @@
         <v>842566</v>
       </c>
       <c r="S33" s="12">
-        <v>823863.77</v>
+        <v>904476.42</v>
       </c>
     </row>
     <row r="34" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2987,7 +2987,7 @@
         <v>1164547</v>
       </c>
       <c r="S34" s="12">
-        <v>1095981.6499999999</v>
+        <v>1177704.95</v>
       </c>
     </row>
     <row r="35" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3046,7 +3046,7 @@
         <v>1616072</v>
       </c>
       <c r="S35" s="12">
-        <v>1489376.46</v>
+        <v>1628860.09</v>
       </c>
     </row>
     <row r="36" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3105,7 +3105,7 @@
         <v>4248266</v>
       </c>
       <c r="S36" s="12">
-        <v>4130947.76</v>
+        <v>4451300.0599999996</v>
       </c>
     </row>
     <row r="37" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3164,7 +3164,7 @@
         <v>4583308</v>
       </c>
       <c r="S37" s="12">
-        <v>4248811.8099999996</v>
+        <v>4638719.5599999996</v>
       </c>
     </row>
     <row r="38" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3223,7 +3223,7 @@
         <v>7770907</v>
       </c>
       <c r="S38" s="12">
-        <v>7916822.1100000003</v>
+        <v>8370831.5800000001</v>
       </c>
     </row>
     <row r="39" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3282,7 +3282,7 @@
         <v>6467038</v>
       </c>
       <c r="S39" s="12">
-        <v>6249284.3799999999</v>
+        <v>6583681.9800000004</v>
       </c>
     </row>
     <row r="40" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3341,7 +3341,7 @@
         <v>6797757</v>
       </c>
       <c r="S40" s="12">
-        <v>7123429.2599999998</v>
+        <v>7651008.04</v>
       </c>
     </row>
     <row r="41" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3400,7 +3400,7 @@
         <v>7102985</v>
       </c>
       <c r="S41" s="12">
-        <v>7020979.2699999996</v>
+        <v>7382996.0899999999</v>
       </c>
     </row>
     <row r="42" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3459,7 +3459,7 @@
         <v>15605360</v>
       </c>
       <c r="S42" s="12">
-        <v>14724194.82</v>
+        <v>15908840.77</v>
       </c>
     </row>
     <row r="43" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3518,7 +3518,7 @@
         <v>88131</v>
       </c>
       <c r="S43" s="10">
-        <v>86365.67</v>
+        <v>88385.54</v>
       </c>
     </row>
     <row r="44" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3577,7 +3577,7 @@
         <v>155500</v>
       </c>
       <c r="S44" s="10">
-        <v>155630.15</v>
+        <v>159135.22</v>
       </c>
       <c r="T44" s="16"/>
     </row>
@@ -3637,7 +3637,7 @@
         <v>205552</v>
       </c>
       <c r="S45" s="10">
-        <v>206388.68</v>
+        <v>207166.13</v>
       </c>
     </row>
     <row r="46" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3696,7 +3696,7 @@
         <v>242452</v>
       </c>
       <c r="S46" s="10">
-        <v>243568.75</v>
+        <v>251706.23999999999</v>
       </c>
       <c r="T46" s="16"/>
     </row>
@@ -3756,7 +3756,7 @@
         <v>426951</v>
       </c>
       <c r="S47" s="10">
-        <v>425482.95</v>
+        <v>429107.57</v>
       </c>
     </row>
     <row r="48" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3815,7 +3815,7 @@
         <v>969064</v>
       </c>
       <c r="S48" s="10">
-        <v>961153.43</v>
+        <v>971315.04</v>
       </c>
     </row>
     <row r="49" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3874,7 +3874,7 @@
         <v>1187092</v>
       </c>
       <c r="S49" s="10">
-        <v>1187092.5900000001</v>
+        <v>1195020.8899999999</v>
       </c>
     </row>
     <row r="50" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3933,7 +3933,7 @@
         <v>1442153</v>
       </c>
       <c r="S50" s="10">
-        <v>1466642.54</v>
+        <v>1472331.13</v>
       </c>
     </row>
     <row r="51" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3992,7 +3992,7 @@
         <v>2183137</v>
       </c>
       <c r="S51" s="10">
-        <v>2173578.39</v>
+        <v>2189777.17</v>
       </c>
     </row>
     <row r="52" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4051,7 +4051,7 @@
         <v>2470833</v>
       </c>
       <c r="S52" s="10">
-        <v>2398853.48</v>
+        <v>2461355.83</v>
       </c>
     </row>
     <row r="53" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4110,7 +4110,7 @@
         <v>3399342</v>
       </c>
       <c r="S53" s="10">
-        <v>3336058.43</v>
+        <v>3386407.26</v>
       </c>
     </row>
     <row r="54" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4169,7 +4169,7 @@
         <v>4553407</v>
       </c>
       <c r="S54" s="10">
-        <v>4570523.9800000004</v>
+        <v>4577366.07</v>
       </c>
       <c r="T54" s="16"/>
     </row>
@@ -4229,7 +4229,7 @@
         <v>6552392</v>
       </c>
       <c r="S55" s="10">
-        <v>6520606.3700000001</v>
+        <v>6557063.9000000004</v>
       </c>
     </row>
     <row r="56" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4288,7 +4288,7 @@
         <v>13891830</v>
       </c>
       <c r="S56" s="10">
-        <v>13816880.529999999</v>
+        <v>14505554.59</v>
       </c>
     </row>
     <row r="57" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4347,7 +4347,7 @@
         <v>18273340</v>
       </c>
       <c r="S57" s="10">
-        <v>18026388.100000001</v>
+        <v>18361604.609999999</v>
       </c>
     </row>
     <row r="58" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4406,7 +4406,7 @@
         <v>26010780</v>
       </c>
       <c r="S58" s="10">
-        <v>26029479.48</v>
+        <v>26749599.43</v>
       </c>
     </row>
     <row r="59" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4465,7 +4465,7 @@
         <v>23687540</v>
       </c>
       <c r="S59" s="10">
-        <v>23583861.52</v>
+        <v>24177749.469999999</v>
       </c>
     </row>
     <row r="60" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4524,7 +4524,7 @@
         <v>26032000</v>
       </c>
       <c r="S60" s="10">
-        <v>26807644.57</v>
+        <v>27796552.98</v>
       </c>
     </row>
     <row r="61" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4583,7 +4583,7 @@
         <v>27282770</v>
       </c>
       <c r="S61" s="10">
-        <v>27334035.09</v>
+        <v>27714647.23</v>
       </c>
     </row>
     <row r="62" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4642,7 +4642,7 @@
         <v>57896250</v>
       </c>
       <c r="S62" s="10">
-        <v>56748874.119999997</v>
+        <v>58063599.710000001</v>
       </c>
     </row>
     <row r="63" spans="1:20" ht="16" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update CoCo+ results with the mean and my lovely MMAILS ;)
</commit_message>
<xml_diff>
--- a/ttp_literature_catABC_results_updated.xlsx
+++ b/ttp_literature_catABC_results_updated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maohammed/Desktop/ttp-dashboard-repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F0C1D8-BB4D-BC4A-AFFC-C83C71754838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB046F97-AF3D-804D-93A2-8ABCD2D1C6F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38400" yWindow="-5500" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1132,7 +1132,7 @@
         <v>3717</v>
       </c>
       <c r="S3" s="8">
-        <v>4100.8</v>
+        <v>4074.8</v>
       </c>
       <c r="T3" s="16"/>
     </row>
@@ -1165,7 +1165,7 @@
         <v>22</v>
       </c>
       <c r="J4" s="8">
-        <v>4881</v>
+        <v>4785</v>
       </c>
       <c r="K4" s="8">
         <v>4389</v>
@@ -1192,7 +1192,7 @@
         <v>4703</v>
       </c>
       <c r="S4" s="8">
-        <v>4911.16</v>
+        <v>4959.7</v>
       </c>
       <c r="T4" s="16"/>
     </row>
@@ -1225,7 +1225,7 @@
         <v>28</v>
       </c>
       <c r="J5" s="8">
-        <v>9632</v>
+        <v>9567</v>
       </c>
       <c r="K5" s="8">
         <v>8813</v>
@@ -1252,7 +1252,7 @@
         <v>8868</v>
       </c>
       <c r="S5" s="8">
-        <v>9680.64</v>
+        <v>9625.4</v>
       </c>
     </row>
     <row r="6" spans="1:24" ht="16" x14ac:dyDescent="0.2">
@@ -1284,7 +1284,7 @@
         <v>33</v>
       </c>
       <c r="J6" s="8">
-        <v>8979</v>
+        <v>8763</v>
       </c>
       <c r="K6" s="8">
         <v>8514</v>
@@ -1311,7 +1311,7 @@
         <v>8314</v>
       </c>
       <c r="S6" s="8">
-        <v>9063.68</v>
+        <v>8702.7000000000007</v>
       </c>
       <c r="T6" s="17"/>
     </row>
@@ -1344,7 +1344,7 @@
         <v>38</v>
       </c>
       <c r="J7" s="8">
-        <v>18702</v>
+        <v>18561</v>
       </c>
       <c r="K7" s="8">
         <v>17474</v>
@@ -1371,7 +1371,7 @@
         <v>17639</v>
       </c>
       <c r="S7" s="8">
-        <v>19164.439999999999</v>
+        <v>18667.099999999999</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="16" x14ac:dyDescent="0.2">
@@ -1403,7 +1403,7 @@
         <v>44</v>
       </c>
       <c r="J8" s="8">
-        <v>28282</v>
+        <v>27453</v>
       </c>
       <c r="K8" s="8">
         <v>26212</v>
@@ -1430,7 +1430,7 @@
         <v>25881</v>
       </c>
       <c r="S8" s="8">
-        <v>28195.53</v>
+        <v>28045.599999999999</v>
       </c>
       <c r="T8" s="17"/>
     </row>
@@ -1463,7 +1463,7 @@
         <v>49</v>
       </c>
       <c r="J9" s="8">
-        <v>51427</v>
+        <v>51120</v>
       </c>
       <c r="K9" s="8">
         <v>49300</v>
@@ -1490,7 +1490,7 @@
         <v>48865</v>
       </c>
       <c r="S9" s="8">
-        <v>50872.11</v>
+        <v>50839.3</v>
       </c>
     </row>
     <row r="10" spans="1:24" ht="16" x14ac:dyDescent="0.2">
@@ -1522,7 +1522,7 @@
         <v>55</v>
       </c>
       <c r="J10" s="8">
-        <v>144426</v>
+        <v>144219</v>
       </c>
       <c r="K10" s="8">
         <v>144219</v>
@@ -1586,7 +1586,7 @@
         <v>60</v>
       </c>
       <c r="J11" s="8">
-        <v>81921</v>
+        <v>81737</v>
       </c>
       <c r="K11" s="8">
         <v>75990</v>
@@ -1613,7 +1613,7 @@
         <v>75804</v>
       </c>
       <c r="S11" s="8">
-        <v>81660.87</v>
+        <v>81348.2</v>
       </c>
       <c r="T11" s="17"/>
       <c r="W11" s="19" t="s">
@@ -1650,7 +1650,7 @@
         <v>65</v>
       </c>
       <c r="J12" s="8">
-        <v>94066</v>
+        <v>93236</v>
       </c>
       <c r="K12" s="8">
         <v>85521</v>
@@ -1677,7 +1677,7 @@
         <v>88330</v>
       </c>
       <c r="S12" s="8">
-        <v>92517.04</v>
+        <v>93215.5</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="16" x14ac:dyDescent="0.2">
@@ -1709,7 +1709,7 @@
         <v>70</v>
       </c>
       <c r="J13" s="8">
-        <v>122902</v>
+        <v>121914</v>
       </c>
       <c r="K13" s="8">
         <v>117456</v>
@@ -1736,7 +1736,7 @@
         <v>112686</v>
       </c>
       <c r="S13" s="8">
-        <v>120744.83</v>
+        <v>122244.5</v>
       </c>
       <c r="T13" s="16"/>
     </row>
@@ -1769,7 +1769,7 @@
         <v>75</v>
       </c>
       <c r="J14" s="8">
-        <v>162321</v>
+        <v>161336</v>
       </c>
       <c r="K14" s="8">
         <v>142158</v>
@@ -1796,7 +1796,7 @@
         <v>148988</v>
       </c>
       <c r="S14" s="8">
-        <v>161191.96</v>
+        <v>161883.5</v>
       </c>
       <c r="T14" s="17"/>
     </row>
@@ -1829,7 +1829,7 @@
         <v>80</v>
       </c>
       <c r="J15" s="8">
-        <v>265322</v>
+        <v>264460</v>
       </c>
       <c r="K15" s="8">
         <v>239048</v>
@@ -1856,7 +1856,7 @@
         <v>248482</v>
       </c>
       <c r="S15" s="8">
-        <v>263543.98</v>
+        <v>262837.2</v>
       </c>
       <c r="T15" s="17"/>
     </row>
@@ -1889,7 +1889,7 @@
         <v>86</v>
       </c>
       <c r="J16" s="8">
-        <v>402199</v>
+        <v>398464</v>
       </c>
       <c r="K16" s="8">
         <v>318077</v>
@@ -1916,7 +1916,7 @@
         <v>367247</v>
       </c>
       <c r="S16" s="8">
-        <v>403684.62</v>
+        <v>403185.8</v>
       </c>
     </row>
     <row r="17" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -1948,7 +1948,7 @@
         <v>91</v>
       </c>
       <c r="J17" s="8">
-        <v>716458</v>
+        <v>714188</v>
       </c>
       <c r="K17" s="8">
         <v>657508</v>
@@ -1975,7 +1975,7 @@
         <v>662940</v>
       </c>
       <c r="S17" s="8">
-        <v>710997.64</v>
+        <v>709726.4</v>
       </c>
       <c r="T17" s="17"/>
     </row>
@@ -2008,7 +2008,7 @@
         <v>96</v>
       </c>
       <c r="J18" s="8">
-        <v>817069</v>
+        <v>809986</v>
       </c>
       <c r="K18" s="8">
         <v>682195</v>
@@ -2035,7 +2035,7 @@
         <v>743146</v>
       </c>
       <c r="S18" s="8">
-        <v>810879.96</v>
+        <v>816606.8</v>
       </c>
     </row>
     <row r="19" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2067,7 +2067,7 @@
         <v>101</v>
       </c>
       <c r="J19" s="8">
-        <v>887033</v>
+        <v>879741</v>
       </c>
       <c r="K19" s="8">
         <v>811069</v>
@@ -2094,7 +2094,7 @@
         <v>813977</v>
       </c>
       <c r="S19" s="8">
-        <v>873102.07</v>
+        <v>881571.7</v>
       </c>
       <c r="T19" s="17"/>
     </row>
@@ -2127,7 +2127,7 @@
         <v>106</v>
       </c>
       <c r="J20" s="8">
-        <v>975930</v>
+        <v>962738</v>
       </c>
       <c r="K20" s="8">
         <v>870796</v>
@@ -2154,7 +2154,7 @@
         <v>871348</v>
       </c>
       <c r="S20" s="8">
-        <v>952282.51</v>
+        <v>964424.6</v>
       </c>
       <c r="T20" s="17"/>
     </row>
@@ -2187,7 +2187,7 @@
         <v>111</v>
       </c>
       <c r="J21" s="8">
-        <v>1088840</v>
+        <v>1082451</v>
       </c>
       <c r="K21" s="8">
         <v>969146</v>
@@ -2214,7 +2214,7 @@
         <v>996820</v>
       </c>
       <c r="S21" s="8">
-        <v>1078267.3799999999</v>
+        <v>1078192.5</v>
       </c>
       <c r="T21" s="17"/>
     </row>
@@ -2247,7 +2247,7 @@
         <v>117</v>
       </c>
       <c r="J22" s="8">
-        <v>1928935</v>
+        <v>1910419</v>
       </c>
       <c r="K22" s="8">
         <v>1785468</v>
@@ -2274,7 +2274,7 @@
         <v>1730997</v>
       </c>
       <c r="S22" s="8">
-        <v>1917935.56</v>
+        <v>1917188.9</v>
       </c>
       <c r="T22" s="16"/>
     </row>
@@ -2307,7 +2307,7 @@
         <v>18</v>
       </c>
       <c r="J23" s="12">
-        <v>22464</v>
+        <v>22290</v>
       </c>
       <c r="K23" s="12">
         <v>21325</v>
@@ -2334,7 +2334,7 @@
         <v>22286</v>
       </c>
       <c r="S23" s="12">
-        <v>22776.92</v>
+        <v>22776.9</v>
       </c>
       <c r="T23" s="16"/>
     </row>
@@ -2367,7 +2367,7 @@
         <v>23</v>
       </c>
       <c r="J24" s="12">
-        <v>45812</v>
+        <v>45662</v>
       </c>
       <c r="K24" s="12">
         <v>39271</v>
@@ -2394,7 +2394,7 @@
         <v>43310</v>
       </c>
       <c r="S24" s="12">
-        <v>46633.18</v>
+        <v>46633.2</v>
       </c>
       <c r="T24" s="17"/>
     </row>
@@ -2427,7 +2427,7 @@
         <v>29</v>
       </c>
       <c r="J25" s="12">
-        <v>61842</v>
+        <v>61702</v>
       </c>
       <c r="K25" s="12">
         <v>56717</v>
@@ -2454,7 +2454,7 @@
         <v>60705</v>
       </c>
       <c r="S25" s="12">
-        <v>61718.36</v>
+        <v>61636.3</v>
       </c>
       <c r="T25" s="16"/>
     </row>
@@ -2487,7 +2487,7 @@
         <v>34</v>
       </c>
       <c r="J26" s="12">
-        <v>61077</v>
+        <v>60814</v>
       </c>
       <c r="K26" s="12">
         <v>59362</v>
@@ -2514,7 +2514,7 @@
         <v>58778</v>
       </c>
       <c r="S26" s="12">
-        <v>61563.32</v>
+        <v>61290.2</v>
       </c>
     </row>
     <row r="27" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2546,7 +2546,7 @@
         <v>39</v>
       </c>
       <c r="J27" s="12">
-        <v>116458</v>
+        <v>116453</v>
       </c>
       <c r="K27" s="12">
         <v>111321</v>
@@ -2573,7 +2573,7 @@
         <v>111728</v>
       </c>
       <c r="S27" s="12">
-        <v>111443.25</v>
+        <v>115547.4</v>
       </c>
       <c r="T27" s="16"/>
     </row>
@@ -2606,7 +2606,7 @@
         <v>45</v>
       </c>
       <c r="J28" s="12">
-        <v>261515</v>
+        <v>260008</v>
       </c>
       <c r="K28" s="12">
         <v>256089</v>
@@ -2633,7 +2633,7 @@
         <v>252294</v>
       </c>
       <c r="S28" s="12">
-        <v>254878.9</v>
+        <v>262488.59999999998</v>
       </c>
     </row>
     <row r="29" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2665,7 +2665,7 @@
         <v>50</v>
       </c>
       <c r="J29" s="12">
-        <v>323123</v>
+        <v>320751</v>
       </c>
       <c r="K29" s="12">
         <v>310993</v>
@@ -2692,7 +2692,7 @@
         <v>303046</v>
       </c>
       <c r="S29" s="12">
-        <v>317580.79999999999</v>
+        <v>309114.09999999998</v>
       </c>
     </row>
     <row r="30" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2724,7 +2724,7 @@
         <v>56</v>
       </c>
       <c r="J30" s="12">
-        <v>372837</v>
+        <v>369270</v>
       </c>
       <c r="K30" s="12">
         <v>332885</v>
@@ -2751,7 +2751,7 @@
         <v>339630</v>
       </c>
       <c r="S30" s="12">
-        <v>350166.13</v>
+        <v>363171.5</v>
       </c>
     </row>
     <row r="31" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2783,7 +2783,7 @@
         <v>61</v>
       </c>
       <c r="J31" s="12">
-        <v>602276</v>
+        <v>599535</v>
       </c>
       <c r="K31" s="12">
         <v>589020</v>
@@ -2810,7 +2810,7 @@
         <v>573980</v>
       </c>
       <c r="S31" s="12">
-        <v>594322.31999999995</v>
+        <v>587545.9</v>
       </c>
     </row>
     <row r="32" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2842,7 +2842,7 @@
         <v>66</v>
       </c>
       <c r="J32" s="12">
-        <v>639843</v>
+        <v>627066</v>
       </c>
       <c r="K32" s="12">
         <v>636725</v>
@@ -2869,7 +2869,7 @@
         <v>603443</v>
       </c>
       <c r="S32" s="12">
-        <v>613270.18000000005</v>
+        <v>618030.1</v>
       </c>
     </row>
     <row r="33" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2901,7 +2901,7 @@
         <v>71</v>
       </c>
       <c r="J33" s="12">
-        <v>927992</v>
+        <v>923681</v>
       </c>
       <c r="K33" s="12">
         <v>842539</v>
@@ -2928,7 +2928,7 @@
         <v>842566</v>
       </c>
       <c r="S33" s="12">
-        <v>904476.42</v>
+        <v>905989.9</v>
       </c>
     </row>
     <row r="34" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -2960,7 +2960,7 @@
         <v>76</v>
       </c>
       <c r="J34" s="12">
-        <v>1205850</v>
+        <v>1201624</v>
       </c>
       <c r="K34" s="12">
         <v>1199138</v>
@@ -2987,7 +2987,7 @@
         <v>1164547</v>
       </c>
       <c r="S34" s="12">
-        <v>1177704.95</v>
+        <v>1197479.3999999999</v>
       </c>
     </row>
     <row r="35" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3019,7 +3019,7 @@
         <v>81</v>
       </c>
       <c r="J35" s="12">
-        <v>1653828</v>
+        <v>1647646</v>
       </c>
       <c r="K35" s="12">
         <v>1635210</v>
@@ -3046,7 +3046,7 @@
         <v>1616072</v>
       </c>
       <c r="S35" s="12">
-        <v>1628860.09</v>
+        <v>1645305</v>
       </c>
     </row>
     <row r="36" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3078,7 +3078,7 @@
         <v>87</v>
       </c>
       <c r="J36" s="12">
-        <v>4485629</v>
+        <v>4466713</v>
       </c>
       <c r="K36" s="12">
         <v>3716735</v>
@@ -3105,7 +3105,7 @@
         <v>4248266</v>
       </c>
       <c r="S36" s="12">
-        <v>4451300.0599999996</v>
+        <v>4434060</v>
       </c>
     </row>
     <row r="37" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3137,7 +3137,7 @@
         <v>92</v>
       </c>
       <c r="J37" s="12">
-        <v>4823625</v>
+        <v>4788987</v>
       </c>
       <c r="K37" s="12">
         <v>4711119</v>
@@ -3164,7 +3164,7 @@
         <v>4583308</v>
       </c>
       <c r="S37" s="12">
-        <v>4638719.5599999996</v>
+        <v>4708331.0999999996</v>
       </c>
     </row>
     <row r="38" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3196,7 +3196,7 @@
         <v>97</v>
       </c>
       <c r="J38" s="12">
-        <v>8343799</v>
+        <v>8229873</v>
       </c>
       <c r="K38" s="12">
         <v>8156575</v>
@@ -3223,7 +3223,7 @@
         <v>7770907</v>
       </c>
       <c r="S38" s="12">
-        <v>8370831.5800000001</v>
+        <v>8321728.0999999996</v>
       </c>
     </row>
     <row r="39" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3255,7 +3255,7 @@
         <v>102</v>
       </c>
       <c r="J39" s="12">
-        <v>6854612</v>
+        <v>6762582</v>
       </c>
       <c r="K39" s="12">
         <v>6659875</v>
@@ -3282,7 +3282,7 @@
         <v>6467038</v>
       </c>
       <c r="S39" s="12">
-        <v>6583681.9800000004</v>
+        <v>6834163.9000000004</v>
       </c>
     </row>
     <row r="40" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3314,7 +3314,7 @@
         <v>107</v>
       </c>
       <c r="J40" s="12">
-        <v>7942036</v>
+        <v>7701890</v>
       </c>
       <c r="K40" s="12">
         <v>7659458</v>
@@ -3341,7 +3341,7 @@
         <v>6797757</v>
       </c>
       <c r="S40" s="12">
-        <v>7651008.04</v>
+        <v>7723011.2000000002</v>
       </c>
     </row>
     <row r="41" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3373,7 +3373,7 @@
         <v>112</v>
       </c>
       <c r="J41" s="12">
-        <v>7582022</v>
+        <v>7457973</v>
       </c>
       <c r="K41" s="12">
         <v>7590024</v>
@@ -3400,7 +3400,7 @@
         <v>7102985</v>
       </c>
       <c r="S41" s="12">
-        <v>7382996.0899999999</v>
+        <v>7513570.2000000002</v>
       </c>
     </row>
     <row r="42" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3432,7 +3432,7 @@
         <v>118</v>
       </c>
       <c r="J42" s="12">
-        <v>16332634</v>
+        <v>16231654</v>
       </c>
       <c r="K42" s="12">
         <v>15766778</v>
@@ -3459,7 +3459,7 @@
         <v>15605360</v>
       </c>
       <c r="S42" s="12">
-        <v>15908840.77</v>
+        <v>16297645.1</v>
       </c>
     </row>
     <row r="43" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3491,7 +3491,7 @@
         <v>19</v>
       </c>
       <c r="J43" s="10">
-        <v>88211</v>
+        <v>87668</v>
       </c>
       <c r="K43" s="10">
         <v>87699</v>
@@ -3518,7 +3518,7 @@
         <v>88131</v>
       </c>
       <c r="S43" s="10">
-        <v>88385.54</v>
+        <v>88385.5</v>
       </c>
     </row>
     <row r="44" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3550,7 +3550,7 @@
         <v>24</v>
       </c>
       <c r="J44" s="10">
-        <v>159112</v>
+        <v>158758</v>
       </c>
       <c r="K44" s="10">
         <v>155585</v>
@@ -3577,7 +3577,7 @@
         <v>155500</v>
       </c>
       <c r="S44" s="10">
-        <v>159135.22</v>
+        <v>159135.20000000001</v>
       </c>
       <c r="T44" s="16"/>
     </row>
@@ -3610,7 +3610,7 @@
         <v>30</v>
       </c>
       <c r="J45" s="10">
-        <v>207902</v>
+        <v>207081</v>
       </c>
       <c r="K45" s="10">
         <v>199507</v>
@@ -3637,7 +3637,7 @@
         <v>205552</v>
       </c>
       <c r="S45" s="10">
-        <v>207166.13</v>
+        <v>207351.4</v>
       </c>
     </row>
     <row r="46" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3669,7 +3669,7 @@
         <v>35</v>
       </c>
       <c r="J46" s="10">
-        <v>249875</v>
+        <v>248508</v>
       </c>
       <c r="K46" s="10">
         <v>242401</v>
@@ -3696,7 +3696,7 @@
         <v>242452</v>
       </c>
       <c r="S46" s="10">
-        <v>251706.23999999999</v>
+        <v>252118</v>
       </c>
       <c r="T46" s="16"/>
     </row>
@@ -3729,7 +3729,7 @@
         <v>40</v>
       </c>
       <c r="J47" s="10">
-        <v>429138</v>
+        <v>429137</v>
       </c>
       <c r="K47" s="10">
         <v>421785</v>
@@ -3756,7 +3756,7 @@
         <v>426951</v>
       </c>
       <c r="S47" s="10">
-        <v>429107.57</v>
+        <v>429181.2</v>
       </c>
     </row>
     <row r="48" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3788,7 +3788,7 @@
         <v>46</v>
       </c>
       <c r="J48" s="10">
-        <v>970343</v>
+        <v>969708</v>
       </c>
       <c r="K48" s="10">
         <v>962450</v>
@@ -3815,7 +3815,7 @@
         <v>969064</v>
       </c>
       <c r="S48" s="10">
-        <v>971315.04</v>
+        <v>971025.4</v>
       </c>
     </row>
     <row r="49" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3847,7 +3847,7 @@
         <v>51</v>
       </c>
       <c r="J49" s="10">
-        <v>1209029</v>
+        <v>1202541</v>
       </c>
       <c r="K49" s="10">
         <v>1196102</v>
@@ -3874,7 +3874,7 @@
         <v>1187092</v>
       </c>
       <c r="S49" s="10">
-        <v>1195020.8899999999</v>
+        <v>1195535.6000000001</v>
       </c>
     </row>
     <row r="50" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3906,7 +3906,7 @@
         <v>57</v>
       </c>
       <c r="J50" s="10">
-        <v>1496922</v>
+        <v>1494506</v>
       </c>
       <c r="K50" s="10">
         <v>1468867</v>
@@ -3933,7 +3933,7 @@
         <v>1442153</v>
       </c>
       <c r="S50" s="10">
-        <v>1472331.13</v>
+        <v>1492328.5</v>
       </c>
     </row>
     <row r="51" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -3965,7 +3965,7 @@
         <v>62</v>
       </c>
       <c r="J51" s="10">
-        <v>2214091</v>
+        <v>2213447</v>
       </c>
       <c r="K51" s="10">
         <v>2201898</v>
@@ -3992,7 +3992,7 @@
         <v>2183137</v>
       </c>
       <c r="S51" s="10">
-        <v>2189777.17</v>
+        <v>2194666.7999999998</v>
       </c>
     </row>
     <row r="52" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4024,7 +4024,7 @@
         <v>67</v>
       </c>
       <c r="J52" s="10">
-        <v>2500736</v>
+        <v>2487396</v>
       </c>
       <c r="K52" s="10">
         <v>2507893</v>
@@ -4051,7 +4051,7 @@
         <v>2470833</v>
       </c>
       <c r="S52" s="10">
-        <v>2461355.83</v>
+        <v>2474627.7999999998</v>
       </c>
     </row>
     <row r="53" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4083,7 +4083,7 @@
         <v>72</v>
       </c>
       <c r="J53" s="10">
-        <v>3501889</v>
+        <v>3496012</v>
       </c>
       <c r="K53" s="10">
         <v>3374021</v>
@@ -4110,7 +4110,7 @@
         <v>3399342</v>
       </c>
       <c r="S53" s="10">
-        <v>3386407.26</v>
+        <v>3459272.3</v>
       </c>
     </row>
     <row r="54" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4142,7 +4142,7 @@
         <v>77</v>
       </c>
       <c r="J54" s="10">
-        <v>4600973</v>
+        <v>4597236</v>
       </c>
       <c r="K54" s="10">
         <v>4618080</v>
@@ -4169,7 +4169,7 @@
         <v>4553407</v>
       </c>
       <c r="S54" s="10">
-        <v>4577366.07</v>
+        <v>4581613.2</v>
       </c>
       <c r="T54" s="16"/>
     </row>
@@ -4202,7 +4202,7 @@
         <v>82</v>
       </c>
       <c r="J55" s="10">
-        <v>6575472</v>
+        <v>6572238</v>
       </c>
       <c r="K55" s="10">
         <v>6545274</v>
@@ -4229,7 +4229,7 @@
         <v>6552392</v>
       </c>
       <c r="S55" s="10">
-        <v>6557063.9000000004</v>
+        <v>6569991.4000000004</v>
       </c>
     </row>
     <row r="56" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4261,7 +4261,7 @@
         <v>88</v>
       </c>
       <c r="J56" s="10">
-        <v>14572352</v>
+        <v>14480550</v>
       </c>
       <c r="K56" s="10">
         <v>13205606</v>
@@ -4288,7 +4288,7 @@
         <v>13891830</v>
       </c>
       <c r="S56" s="10">
-        <v>14505554.59</v>
+        <v>14419727.199999999</v>
       </c>
     </row>
     <row r="57" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4320,7 +4320,7 @@
         <v>93</v>
       </c>
       <c r="J57" s="10">
-        <v>18569005</v>
+        <v>18381502</v>
       </c>
       <c r="K57" s="10">
         <v>18510201</v>
@@ -4347,7 +4347,7 @@
         <v>18273340</v>
       </c>
       <c r="S57" s="10">
-        <v>18361604.609999999</v>
+        <v>18487869.5</v>
       </c>
     </row>
     <row r="58" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4379,7 +4379,7 @@
         <v>98</v>
       </c>
       <c r="J58" s="10">
-        <v>26728716</v>
+        <v>26404068</v>
       </c>
       <c r="K58" s="10">
         <v>26456558</v>
@@ -4406,7 +4406,7 @@
         <v>26010780</v>
       </c>
       <c r="S58" s="10">
-        <v>26749599.43</v>
+        <v>26561314.5</v>
       </c>
     </row>
     <row r="59" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4438,7 +4438,7 @@
         <v>103</v>
       </c>
       <c r="J59" s="10">
-        <v>24361366</v>
+        <v>24152244</v>
       </c>
       <c r="K59" s="10">
         <v>23906422</v>
@@ -4465,7 +4465,7 @@
         <v>23687540</v>
       </c>
       <c r="S59" s="10">
-        <v>24177749.469999999</v>
+        <v>24240428.699999999</v>
       </c>
     </row>
     <row r="60" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4497,7 +4497,7 @@
         <v>108</v>
       </c>
       <c r="J60" s="10">
-        <v>27665466</v>
+        <v>27462464</v>
       </c>
       <c r="K60" s="10">
         <v>27209683</v>
@@ -4524,7 +4524,7 @@
         <v>26032000</v>
       </c>
       <c r="S60" s="10">
-        <v>27796552.98</v>
+        <v>27546552.5</v>
       </c>
     </row>
     <row r="61" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4556,7 +4556,7 @@
         <v>113</v>
       </c>
       <c r="J61" s="10">
-        <v>27951166</v>
+        <v>27766028</v>
       </c>
       <c r="K61" s="10">
         <v>27872957</v>
@@ -4583,7 +4583,7 @@
         <v>27282770</v>
       </c>
       <c r="S61" s="10">
-        <v>27714647.23</v>
+        <v>27910428.5</v>
       </c>
     </row>
     <row r="62" spans="1:20" ht="16" x14ac:dyDescent="0.2">
@@ -4615,7 +4615,7 @@
         <v>119</v>
       </c>
       <c r="J62" s="10">
-        <v>58900443</v>
+        <v>58680600</v>
       </c>
       <c r="K62" s="10">
         <v>58147460</v>
@@ -4642,7 +4642,7 @@
         <v>57896250</v>
       </c>
       <c r="S62" s="10">
-        <v>58063599.710000001</v>
+        <v>58935700.600000001</v>
       </c>
     </row>
     <row r="63" spans="1:20" ht="16" x14ac:dyDescent="0.2">

</xml_diff>